<commit_message>
Sample report: commentary follows the structure of the real report
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FE233U4YTNJntBW99dBEpw
</commit_message>
<xml_diff>
--- a/analysis/sample-ad-report.xlsx
+++ b/analysis/sample-ad-report.xlsx
@@ -9205,415 +9205,381 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="95" customWidth="1" min="1" max="1"/>
+    <col width="150" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Commentary by portfolio (demo data, 2026-07 to 2026-09, September is partial)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Tiers: MQL rate Good &gt;= 70%, Medium 60-70%, Low &lt; 60%. Won/MQL Strong &gt;= 40%, Average 15-40%, Weak &lt; 15%. Fewer than 10 leads = small sample.</t>
+          <t>Commentary by portfolio (demo data, July-September 2026, September is a partial month)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>SECTION 1: Lead volume and quality (Volume + MQL rate)</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tiers: MQL rate Good &gt;= 70%, Medium 60-70%, Low &lt; 60%. Won/MQL Strong &gt;= 40%, Average 20-40%, Weak &lt; 20%. Fewer than 10 leads (or MQLs) = small sample.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Portfolio</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Lead</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>MQL</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>MQL rate</t>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SECTION 1: Lead volume + quality (Volume + MQL rate)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>58</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>84.5% (Good)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>72.9% (Good)</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Overview of the 3 portfolios (July-September):</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Specialist</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>10</v>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>MQL</t>
+        </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>66.7% (Medium)</t>
+          <t>MQL rate</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>58</v>
+      </c>
+      <c r="C10" t="n">
+        <v>49</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>84.5% (Good, highest)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Advanced: 58 leads in total. MQL rate by month: 78.3% (Good) -&gt; 87.1% (Good) -&gt; 100.0% (Good)</t>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>48</v>
+      </c>
+      <c r="C11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>72.9% (Good)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course D - Advanced: 27 leads, MQL 85.2% (Good)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Combo: Course A + Course C: 21 leads, MQL 85.7% (Good)</t>
+          <t>Specialist</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>15</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>66.7% (Medium, lowest)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course C - Advanced: 10 leads, MQL 80.0% (Good)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Advanced — largest volume, quality improving month after month</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Foundation: 48 leads in total. MQL rate by month: 77.8% (Good) -&gt; 57.1% (Low) -&gt; 85.7% (Good)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course A - Foundation: 23 leads, MQL 69.6% (Medium)</t>
+          <t>MQL rate rises every month: 78.3% (Good) → 87.1% (Good) → 100% (Good) — the only portfolio that improves quality month after month (September is a small sample).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course B - Foundation: 17 leads, MQL 64.7% (Medium)</t>
+          <t>Course D - Advanced: 27 leads, MQL 85.2% — Good — biggest volume in Advanced, and quality is good.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course F - Short course: 8 leads, MQL 100.0% (Good) - small sample, read with care</t>
+          <t>Combo: Course A + Course C: 21 leads, MQL 85.7% — Good — best MQL rate of all courses with enough volume.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Specialist: 15 leads in total. MQL rate by month: 70.0% (Good) -&gt; 50.0% (Low) -&gt; 100.0% (Good)</t>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Course C - Advanced: 10 leads, MQL 80% — Good.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course E - Specialist: 9 leads, MQL 66.7% (Medium) - small sample, read with care</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Program G - Professional: 6 leads, MQL 66.7% (Medium) - small sample, read with care</t>
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Foundation — mid-sized volume, quality stays around the middle</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>SECTION 2: Closing ability (Won / MQL)</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MQL rate moves up and down: 77.8% (Good) → 57.1% (Low) → 85.7% (Good) (September is a small sample).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Course A - Foundation: 23 leads, MQL 69.6% — Medium — biggest volume in Foundation, but quality is only medium.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Portfolio</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>MQL</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Won</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Won/MQL</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Course B - Foundation: 17 leads, MQL 64.7% — Medium — lowest MQL rate of all courses with enough volume.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>44.9% (Strong)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="C29" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>14.3% (Weak)</t>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Course F - Short course: 8 leads, MQL 100% — Good — only 8 leads, the sample is too small.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Specialist</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="C30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>0.0% (Weak)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
+          <t>Specialist — smallest volume, lowest quality of the portfolios, read conclusions with care</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course D - Advanced: 23 MQL -&gt; 10 won (43.5%, Strong)</t>
+          <t>MQL rate moves up and down: 70% (Good) → 50% (Low) → 100% (Good) (September is a small sample).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Combo: Course A + Course C: 18 MQL -&gt; 8 won (44.4%, Strong)</t>
+          <t>Course E - Specialist: 9 leads, MQL 66.7% — Medium — only 9 leads, the sample is too small.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course C - Advanced: 8 MQL -&gt; 4 won (50.0%, Strong) - small sample</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
+          <t>Program G - Professional: 6 leads, MQL 66.7% — Medium — only 6 leads, the sample is too small.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course A - Foundation: 16 MQL -&gt; 1 won (6.2%, Weak)</t>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SECTION 2: Closing ability (Won / MQL)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course B - Foundation: 11 MQL -&gt; 2 won (18.2%, Average)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course F - Short course: 8 MQL -&gt; 2 won (25.0%, Average) - small sample</t>
+          <t>Overview of the 3 portfolios (July-September):</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>MQL</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Won</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Won/MQL</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Specialist</t>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>49</v>
+      </c>
+      <c r="C42" t="n">
+        <v>22</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>44.9% (Strong, highest)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course E - Specialist: 6 MQL -&gt; 0 won (0.0%, Weak) - small sample</t>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>35</v>
+      </c>
+      <c r="C43" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>14.3% (Weak)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Program G - Professional: 4 MQL -&gt; 0 won (0.0%, Weak) - small sample</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
+          <t>Specialist</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>10</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0% (Weak, lowest)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Biggest leak in absolute numbers (MQLs that did not close)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course A - Foundation (Foundation): 16 MQL, only 1 won (6.2%), 15 MQLs lost</t>
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Advanced — closes best of the 3 portfolios</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course D - Advanced (Advanced): 23 MQL, only 10 won (43.5%), 13 MQLs lost</t>
+          <t>Course C - Advanced: 8 MQL → 4 won (50%) — strong — small sample.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Combo: Course A + Course C (Advanced): 18 MQL, only 8 won (44.4%), 10 MQLs lost</t>
+          <t>Combo: Course A + Course C: 18 MQL → 8 won (44.4%) — strong — best closing of all courses with enough volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Course D - Advanced: 23 MQL → 10 won (43.5%) — strong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Foundation — average closing</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Course F - Short course: 8 MQL → 2 won (25%) — average — small sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Course B - Foundation: 11 MQL → 2 won (18.2%) — weak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Course A - Foundation: 16 MQL → 1 won (6.2%) — weak — worst closing of all courses with enough volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Specialist — weakest closing, almost no lead from ads is won</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Course E - Specialist: 6 MQL → 0 won (0%) — weak — small sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Program G - Professional: 4 MQL → 0 won (0%) — weak — small sample.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sample report: commentary follows the real report structure, top 10 ad rows
* Sample report: show the top 10 ad rows in the Markdown version

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FE233U4YTNJntBW99dBEpw

* Sample report: commentary follows the structure of the real report

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FE233U4YTNJntBW99dBEpw

---------

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/sample-ad-report.xlsx
+++ b/analysis/sample-ad-report.xlsx
@@ -9205,415 +9205,381 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="95" customWidth="1" min="1" max="1"/>
+    <col width="150" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Commentary by portfolio (demo data, 2026-07 to 2026-09, September is partial)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Tiers: MQL rate Good &gt;= 70%, Medium 60-70%, Low &lt; 60%. Won/MQL Strong &gt;= 40%, Average 15-40%, Weak &lt; 15%. Fewer than 10 leads = small sample.</t>
+          <t>Commentary by portfolio (demo data, July-September 2026, September is a partial month)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>SECTION 1: Lead volume and quality (Volume + MQL rate)</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tiers: MQL rate Good &gt;= 70%, Medium 60-70%, Low &lt; 60%. Won/MQL Strong &gt;= 40%, Average 20-40%, Weak &lt; 20%. Fewer than 10 leads (or MQLs) = small sample.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Portfolio</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Lead</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>MQL</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>MQL rate</t>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>SECTION 1: Lead volume + quality (Volume + MQL rate)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>58</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>84.5% (Good)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>48</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>72.9% (Good)</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Overview of the 3 portfolios (July-September):</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Specialist</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>10</v>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>MQL</t>
+        </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>66.7% (Medium)</t>
+          <t>MQL rate</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>58</v>
+      </c>
+      <c r="C10" t="n">
+        <v>49</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>84.5% (Good, highest)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Advanced: 58 leads in total. MQL rate by month: 78.3% (Good) -&gt; 87.1% (Good) -&gt; 100.0% (Good)</t>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>48</v>
+      </c>
+      <c r="C11" t="n">
+        <v>35</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>72.9% (Good)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course D - Advanced: 27 leads, MQL 85.2% (Good)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Combo: Course A + Course C: 21 leads, MQL 85.7% (Good)</t>
+          <t>Specialist</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>15</v>
+      </c>
+      <c r="C12" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>66.7% (Medium, lowest)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course C - Advanced: 10 leads, MQL 80.0% (Good)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Advanced — largest volume, quality improving month after month</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Foundation: 48 leads in total. MQL rate by month: 77.8% (Good) -&gt; 57.1% (Low) -&gt; 85.7% (Good)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course A - Foundation: 23 leads, MQL 69.6% (Medium)</t>
+          <t>MQL rate rises every month: 78.3% (Good) → 87.1% (Good) → 100% (Good) — the only portfolio that improves quality month after month (September is a small sample).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course B - Foundation: 17 leads, MQL 64.7% (Medium)</t>
+          <t>Course D - Advanced: 27 leads, MQL 85.2% — Good — biggest volume in Advanced, and quality is good.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course F - Short course: 8 leads, MQL 100.0% (Good) - small sample, read with care</t>
+          <t>Combo: Course A + Course C: 21 leads, MQL 85.7% — Good — best MQL rate of all courses with enough volume.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Specialist: 15 leads in total. MQL rate by month: 70.0% (Good) -&gt; 50.0% (Low) -&gt; 100.0% (Good)</t>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Course C - Advanced: 10 leads, MQL 80% — Good.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course E - Specialist: 9 leads, MQL 66.7% (Medium) - small sample, read with care</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Program G - Professional: 6 leads, MQL 66.7% (Medium) - small sample, read with care</t>
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Foundation — mid-sized volume, quality stays around the middle</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>SECTION 2: Closing ability (Won / MQL)</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>MQL rate moves up and down: 77.8% (Good) → 57.1% (Low) → 85.7% (Good) (September is a small sample).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Course A - Foundation: 23 leads, MQL 69.6% — Medium — biggest volume in Foundation, but quality is only medium.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Portfolio</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>MQL</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>Won</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Won/MQL</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Course B - Foundation: 17 leads, MQL 64.7% — Medium — lowest MQL rate of all courses with enough volume.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>44.9% (Strong)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n">
-        <v>35</v>
-      </c>
-      <c r="C29" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>14.3% (Weak)</t>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Course F - Short course: 8 leads, MQL 100% — Good — only 8 leads, the sample is too small.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Specialist</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="C30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>0.0% (Weak)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
+          <t>Specialist — smallest volume, lowest quality of the portfolios, read conclusions with care</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Advanced</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course D - Advanced: 23 MQL -&gt; 10 won (43.5%, Strong)</t>
+          <t>MQL rate moves up and down: 70% (Good) → 50% (Low) → 100% (Good) (September is a small sample).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Combo: Course A + Course C: 18 MQL -&gt; 8 won (44.4%, Strong)</t>
+          <t>Course E - Specialist: 9 leads, MQL 66.7% — Medium — only 9 leads, the sample is too small.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course C - Advanced: 8 MQL -&gt; 4 won (50.0%, Strong) - small sample</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
+          <t>Program G - Professional: 6 leads, MQL 66.7% — Medium — only 6 leads, the sample is too small.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course A - Foundation: 16 MQL -&gt; 1 won (6.2%, Weak)</t>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>SECTION 2: Closing ability (Won / MQL)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course B - Foundation: 11 MQL -&gt; 2 won (18.2%, Average)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course F - Short course: 8 MQL -&gt; 2 won (25.0%, Average) - small sample</t>
+          <t>Overview of the 3 portfolios (July-September):</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Portfolio</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>MQL</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Won</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Won/MQL</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Specialist</t>
+          <t>Advanced</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>49</v>
+      </c>
+      <c r="C42" t="n">
+        <v>22</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>44.9% (Strong, highest)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course E - Specialist: 6 MQL -&gt; 0 won (0.0%, Weak) - small sample</t>
+          <t>Foundation</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>35</v>
+      </c>
+      <c r="C43" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>14.3% (Weak)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Program G - Professional: 4 MQL -&gt; 0 won (0.0%, Weak) - small sample</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
+          <t>Specialist</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>10</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>0% (Weak, lowest)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Biggest leak in absolute numbers (MQLs that did not close)</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   - Course A - Foundation (Foundation): 16 MQL, only 1 won (6.2%), 15 MQLs lost</t>
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>Advanced — closes best of the 3 portfolios</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Course D - Advanced (Advanced): 23 MQL, only 10 won (43.5%), 13 MQLs lost</t>
+          <t>Course C - Advanced: 8 MQL → 4 won (50%) — strong — small sample.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Combo: Course A + Course C (Advanced): 18 MQL, only 8 won (44.4%), 10 MQLs lost</t>
+          <t>Combo: Course A + Course C: 18 MQL → 8 won (44.4%) — strong — best closing of all courses with enough volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Course D - Advanced: 23 MQL → 10 won (43.5%) — strong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>Foundation — average closing</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Course F - Short course: 8 MQL → 2 won (25%) — average — small sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Course B - Foundation: 11 MQL → 2 won (18.2%) — weak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Course A - Foundation: 16 MQL → 1 won (6.2%) — weak — worst closing of all courses with enough volume.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Specialist — weakest closing, almost no lead from ads is won</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Course E - Specialist: 6 MQL → 0 won (0%) — weak — small sample.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Program G - Professional: 4 MQL → 0 won (0%) — weak — small sample.</t>
         </is>
       </c>
     </row>

</xml_diff>